<commit_message>
Set BESS capex to 100 k€/MWh on built MWh in the Bora and non-delivery models
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011Cy4jTfjKbxPfMRQvaZwVT
</commit_message>
<xml_diff>
--- a/projects/bora_nondelivery/out/Bora_NonDelivery.xlsx
+++ b/projects/bora_nondelivery/out/Bora_NonDelivery.xlsx
@@ -2596,12 +2596,12 @@
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>EUR k/MW</t>
+          <t>EUR k/MWh</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Bora model Inputs (user 12-Oct-26)</t>
+          <t>Bora model Inputs (user 15-Oct-26)</t>
         </is>
       </c>
       <c r="F39" s="17">
@@ -2609,7 +2609,7 @@
         <v/>
       </c>
       <c r="H39" s="30" t="n">
-        <v>240</v>
+        <v>100</v>
       </c>
     </row>
     <row r="40">
@@ -3119,7 +3119,7 @@
         <v/>
       </c>
       <c r="H63" s="30" t="n">
-        <v>155571.1355981859</v>
+        <v>163950.6913103223</v>
       </c>
     </row>
     <row r="64">
@@ -8875,7 +8875,7 @@
         </is>
       </c>
       <c r="E34" s="17">
-        <f>In_BESS_Capex*$E14</f>
+        <f>In_BESS_Capex*$F14</f>
         <v/>
       </c>
       <c r="F34" s="17">

</xml_diff>